<commit_message>
more inputs on the advanced tab, download button, minor changes throughout
</commit_message>
<xml_diff>
--- a/advanced.xlsx
+++ b/advanced.xlsx
@@ -5,16 +5,21 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aheller\Documents\GitHub\TEA.CART\inst\app\www\static_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aheller\Dropbox\CS\3 - Current Projects\TEA-CART again\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75C34ED9-E312-4782-ABC0-4502869C7859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B619F310-C6DA-4096-873D-880A99A53A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A33ACDFD-014A-4B2F-8FAD-02B00287D07F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{A33ACDFD-014A-4B2F-8FAD-02B00287D07F}"/>
   </bookViews>
   <sheets>
     <sheet name="ev_forecast" sheetId="1" r:id="rId1"/>
     <sheet name="vmt_forecast" sheetId="2" r:id="rId2"/>
+    <sheet name="onroad_fuel_tech_frac" sheetId="3" r:id="rId3"/>
+    <sheet name="pass_rail" sheetId="4" r:id="rId4"/>
+    <sheet name="freight_rail" sheetId="5" r:id="rId5"/>
+    <sheet name="construction" sheetId="6" r:id="rId6"/>
+    <sheet name="fuel_apportionment" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="38">
   <si>
     <t>Custom EV Baseline</t>
   </si>
@@ -64,6 +69,93 @@
   </si>
   <si>
     <t>Mode</t>
+  </si>
+  <si>
+    <t>Onroad Public Transit - Fuel Technology Fraction</t>
+  </si>
+  <si>
+    <t>Bus</t>
+  </si>
+  <si>
+    <t>Diesel</t>
+  </si>
+  <si>
+    <t>CNG</t>
+  </si>
+  <si>
+    <t>Electric</t>
+  </si>
+  <si>
+    <t>Demand Response</t>
+  </si>
+  <si>
+    <t>Gasoline</t>
+  </si>
+  <si>
+    <t>Commuter Bus</t>
+  </si>
+  <si>
+    <t>Passenger Rail</t>
+  </si>
+  <si>
+    <t>Amtrak</t>
+  </si>
+  <si>
+    <t>Average Trip Length (mi)</t>
+  </si>
+  <si>
+    <t>Commuter Rail</t>
+  </si>
+  <si>
+    <t>Heavy Rail</t>
+  </si>
+  <si>
+    <t>Light Rail</t>
+  </si>
+  <si>
+    <t>Freight Rail</t>
+  </si>
+  <si>
+    <t>Growth Rate</t>
+  </si>
+  <si>
+    <t>Energy Intensity (BTU / ton-mile)</t>
+  </si>
+  <si>
+    <t>Construction and Maintenance</t>
+  </si>
+  <si>
+    <t>Annual MT CO2e</t>
+  </si>
+  <si>
+    <t>Direct Emissions</t>
+  </si>
+  <si>
+    <t>Upstream Emissions</t>
+  </si>
+  <si>
+    <t>Fuel Apportionment</t>
+  </si>
+  <si>
+    <t>% PHEV Miles Driven on Electricity</t>
+  </si>
+  <si>
+    <t>Fuel</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Emissions Type</t>
+  </si>
+  <si>
+    <t>Mode/Service</t>
+  </si>
+  <si>
+    <t>Variable</t>
+  </si>
+  <si>
+    <t>Energy Source (Diesel/Electric)</t>
   </si>
 </sst>
 </file>
@@ -676,4 +768,353 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25257236-E1FA-4834-ADF1-B3765F20D5D9}">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="5" width="20.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2522103F-ECFF-4805-B93D-4D869DA1F36C}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="26.28515625" customWidth="1"/>
+    <col min="2" max="2" width="33.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3">
+        <v>198.354755374798</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B78C60D9-A139-46A4-8FEC-CDF7BFD9E702}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="30.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3">
+        <v>6.8639406622490462E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4">
+        <v>297.57986556812102</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63FEE0DB-0F72-4444-98D4-482C19D3929A}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="26.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33CCAFE3-0A10-4A51-A2ED-4041AAB9D655}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="30.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>0.54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>0.54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>0.1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>